<commit_message>
Propose CV-JD pairs with label overrides and package rater kits
- make_pairs: 24 GOLD40 CVs x 2 JDs (same/other track), share-based JD choice,
  load caps for long JDs, at least 2 pairs per JD, split by CV (8 dev / 16 test).
- cv_track_overrides.csv wins over the heuristic track; cv_track_review.csv lists
  all 40 GOLD40 CVs for the PDF check.
- package_rater: locked workbook, CV PDFs named by id and a 2-page guide per rater;
  never ships pairs.csv, gold or model output. Workbook builder gains --split.
- Input hashes fold CRLF to LF so Windows copies match the git checkout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -34,7 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TIEN_DO'!$A$1:$G$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'TIEN_DO'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'DANH_MUC'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'META'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'META'!$A$1:$B$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'META'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -797,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -901,57 +901,69 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>pair_count</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>3</v>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>criterion_rows</t>
+          <t>pair_count</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>requirement_rows</t>
+          <t>criterion_rows</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>locked</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="b">
-        <v>0</v>
+          <t>requirement_rows</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>locked</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>2026-10-13T00:00:00Z</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Tell raters how to map CV sections that are not in the evidence list
A separate "Ngoại ngữ" section maps to skills (scored certificates to
certifications); toan_bo_cv stays reserved for C1 and C7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -634,152 +634,159 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Với C1 và C7 (hình thức, ATS), chọn muc_bang_chung = toan_bo_cv và mô tả ngắn điều quan sát được ở cột trich_dan.</t>
+          <t>• Với C1 và C7 (hình thức, ATS), chọn muc_bang_chung = toan_bo_cv và mô tả ngắn điều quan sát được ở cột trich_dan. Không dùng toan_bo_cv cho trích dẫn thông thường.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>• Mục trong CV có tên khác danh sách thì chọn mục tương ứng: Ngoại ngữ → skills (chứng chỉ có điểm như TOEIC, IELTS → certifications); Mục tiêu, Giới thiệu, Profile → summary; Thực tập, Công việc → experience; Đồ án → projects; Giải thưởng, Thành tích → awards; Hoạt động, CLB, Tình nguyện → activities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
+          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
+          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>• missing: Không thấy trong CV.</t>
+          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>• missing: Không thấy trong CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
+          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
+          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Lưu ý</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>• Nếu mô tả neo không đủ để quyết định, ghi lại ở cột ghi_chu để thảo luận khi phân xử.</t>
         </is>

</xml_diff>

<commit_message>
Rate from the CV text only and settle GitHub links against Git
Raters do not open links. A GitHub link tied to a project counts as Git
used (met); a profile link in the contact block counts as mentioned_only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -646,147 +646,161 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>• Chỉ chấm theo nội dung CV; không mở link GitHub, portfolio hay demo. Link chỉ tính như một dòng chữ trong CV.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
+          <t>• Link GitHub với yêu cầu Git: link gắn với một dự án cụ thể → met (projects); chỉ có link hồ sơ ở phần liên hệ → mentioned_only (personal_info); Git/GitHub chỉ ghi trong mục kỹ năng → mentioned_only (skills).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
+          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
+          <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>• missing: Không thấy trong CV.</t>
+          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
+          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>• missing: Không thấy trong CV.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
+          <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
+          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
+          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Lưu ý</t>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
+          <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lưu ý</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>• Nếu mô tả neo không đủ để quyết định, ghi lại ở cột ghi_chu để thảo luận khi phân xử.</t>
         </is>

</xml_diff>

<commit_message>
Guide raters on requirement levels, other abilities and alternatives
Ignore proficiency words; a different ability in the same area (reading vs
English communication) is missing with a note; one alternative is enough;
skills only implied stay unclear.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -655,152 +655,159 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>• Yêu cầu JD: bỏ qua mức độ (thành thạo, cơ bản); CV nêu một khả năng khác cùng lĩnh vực → missing kèm ghi chú (JD cần giao tiếp tiếng Anh, CV chỉ đọc tài liệu); yêu cầu có 'A hoặc B' → có một lựa chọn là đủ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>• Link GitHub với yêu cầu Git: link gắn với một dự án cụ thể → met (projects); chỉ có link hồ sơ ở phần liên hệ → mentioned_only (personal_info); Git/GitHub chỉ ghi trong mục kỹ năng → mentioned_only (skills).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
+          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
+          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>• missing: Không thấy trong CV.</t>
+          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>• missing: Không thấy trong CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
+          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
+          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Lưu ý</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>• Nếu mô tả neo không đủ để quyết định, ghi lại ở cột ghi_chu để thảo luận khi phân xử.</t>
         </is>

</xml_diff>

<commit_message>
Count directly implied skills as present; keep loose associations unclear
A framework that cannot be used without the required skill (Spring Boot ->
Java, a FastAPI backend -> REST API) now counts like the skill itself, with
a note; looser links (Docker -> Linux) stay unclear. Replaces the earlier
"implied means unclear" rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -662,152 +662,159 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>• Bao hàm trực tiếp (Spring Boot → Java, FastAPI backend → REST API…) → xem như có kỹ năng, ghi chú đã suy ra từ đâu; liên quan lỏng (Docker → Linux, Git → CI/CD) → unclear. Danh sách đầy đủ trong 00_DOC_TRUOC.docx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>• Link GitHub với yêu cầu Git: link gắn với một dự án cụ thể → met (projects); chỉ có link hồ sơ ở phần liên hệ → mentioned_only (personal_info); Git/GitHub chỉ ghi trong mục kỹ năng → mentioned_only (skills).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
+          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
+          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• missing: Không thấy trong CV.</t>
+          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>• missing: Không thấy trong CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
+          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
+          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Lưu ý</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>• Nếu mô tả neo không đủ để quyết định, ghi lại ở cột ghi_chu để thảo luận khi phân xử.</t>
         </is>

</xml_diff>

<commit_message>
Add rater rules for the ambiguous cases seen in the pilot
Self-claimed experience, languages and soft skills, soft-skill synonyms,
same-kind tools with other names, tool categories, domain requirements,
missing_in_cv for absent content, the C8 share bands and contiguous quotes.
Rules are general so the second rater learns no pair-specific answers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
+++ b/downstream/templates/CV_JD_RATING_TEMPLATE_v1_DEMO.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -669,152 +669,159 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>• Các trường hợp khác (câu tự nhận kinh nghiệm, ngoại ngữ và kỹ năng mềm, công cụ khác tên, lĩnh vực, cách tính C8, khi nào dùng missing_in_cv) xem mục 'Một số trường hợp khó' trong 00_DOC_TRUOC.docx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>• Link GitHub với yêu cầu Git: link gắn với một dự án cụ thể → met (projects); chỉ có link hồ sơ ở phần liên hệ → mentioned_only (personal_info); Git/GitHub chỉ ghi trong mục kỹ năng → mentioned_only (skills).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Trạng thái tiêu chí (cột trang_thai ở TIEU_CHI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
+          <t>• scored: Đã chấm 0–4 theo mô tả neo.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+          <t>• missing_in_cv: PDF đọc được nhưng CV không có nội dung cho tiêu chí này. Điểm bắt buộc là 0.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>• not_applicable: Tiêu chí không áp dụng cho vị trí theo quy tắc đã chốt. Bỏ trống điểm và ghi lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>• unreadable: Không đọc chắc được phần nội dung liên quan trong PDF (mờ, vỡ font, mất trang). Bỏ trống điểm.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Trạng thái yêu cầu JD (cột trang_thai ở YEU_CAU_JD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
+          <t>• met: CV có bằng chứng sử dụng trong dự án, kinh nghiệm hoặc chứng chỉ.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• missing: Không thấy trong CV.</t>
+          <t>• mentioned_only: Chỉ xuất hiện trong danh sách kỹ năng hoặc mục tiêu, không có ngữ cảnh sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>• missing: Không thấy trong CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>• unclear: Có dấu hiệu liên quan nhưng không đủ để quyết định; ghi lý do ở cột ghi chú.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Mức phù hợp tổng thể (cột muc_phu_hop ở TONG_THE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
+          <t>• 1 · Không phù hợp: thiếu phần lớn yêu cầu cốt lõi.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
+          <t>• 2 · Ít phù hợp: chỉ đáp ứng vài yêu cầu, thiếu nền tảng chính.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+          <t>• 3 · Phù hợp một phần: có nền tảng nhưng thiếu vài yêu cầu bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>• 4 · Phù hợp: đáp ứng hầu hết yêu cầu bắt buộc có bằng chứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>• 5 · Rất phù hợp: đáp ứng gần đủ yêu cầu bắt buộc và nhiều yêu cầu ưu tiên, minh chứng mạnh.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Lưu ý</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
+          <t>• Không chấm theo tên, giới tính, ảnh, quê quán, trường học hay thông tin cá nhân. Thông tin liên hệ không dùng để cho điểm.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+          <t>• Không thêm, xóa hay đổi thứ tự dòng; không đổi tên sheet hoặc tiêu đề cột. Chỉ nhập ở cột trắng; cột màu xám là cố định.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>• File chứa trích dẫn từ CV thật: chỉ lưu trong thư mục nhóm đã thống nhất, không gửi qua kênh công khai, không đưa lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>• Nếu mô tả neo không đủ để quyết định, ghi lại ở cột ghi_chu để thảo luận khi phân xử.</t>
         </is>

</xml_diff>